<commit_message>
Pierre Verweij left the board in November (last year) – remove from board member listing
</commit_message>
<xml_diff>
--- a/data/roster.xlsx
+++ b/data/roster.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schaej17\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB09C49C-6EDD-4843-8BC3-95AA5EC8443E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E8132E-91E2-4598-8168-509DC2AEE278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="120" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020 Roster" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,21 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2020 Roster'!$A$1:$T$37</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -982,6 +993,9 @@
         <v>47</v>
       </c>
       <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Alessandro and Nikki as the BBS SR and BBS NextGen representatives, respectively
</commit_message>
<xml_diff>
--- a/data/roster.xlsx
+++ b/data/roster.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schaej17\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E8132E-91E2-4598-8168-509DC2AEE278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8704BA3-7F55-4E96-B61C-52E174A1FF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020 Roster" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2020 Roster'!$A$1:$T$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2020 Roster'!$A$1:$T$38</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="109">
   <si>
     <t>Kaspar</t>
   </si>
@@ -305,9 +305,6 @@
     <t>ottavia.prunas@unibas.ch</t>
   </si>
   <si>
-    <t>University Hospital of Basel</t>
-  </si>
-  <si>
     <t>Markus</t>
   </si>
   <si>
@@ -345,6 +342,30 @@
   </si>
   <si>
     <t>marisabacchi@gmail.com</t>
+  </si>
+  <si>
+    <t>Nikki.Rommers@usb.ch</t>
+  </si>
+  <si>
+    <t>Rommers</t>
+  </si>
+  <si>
+    <t>Nikki</t>
+  </si>
+  <si>
+    <t>University Hospital Basel</t>
+  </si>
+  <si>
+    <t>Alessandro.Previtali@bms.com</t>
+  </si>
+  <si>
+    <t>Alessandro</t>
+  </si>
+  <si>
+    <t>Previtali</t>
+  </si>
+  <si>
+    <t>SR representative</t>
   </si>
 </sst>
 </file>
@@ -395,7 +416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -410,6 +431,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -726,7 +748,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:T26"/>
+  <dimension ref="A1:T28"/>
   <sheetFormatPr defaultColWidth="101.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
@@ -805,10 +827,10 @@
         <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E4" s="2">
         <v>1</v>
@@ -970,7 +992,7 @@
         <v>13</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E13" s="2">
         <v>1</v>
@@ -1018,16 +1040,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>61</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E16" s="1"/>
       <c r="G16" s="2" t="s">
@@ -1133,12 +1155,15 @@
         <v>86</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E22" s="2">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2">
         <v>1</v>
       </c>
       <c r="G22" s="2" t="s">
@@ -1147,30 +1172,33 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="E23" s="2">
         <v>1</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>99</v>
@@ -1181,16 +1209,16 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E25" s="2">
         <v>1</v>
@@ -1198,13 +1226,13 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>91</v>
+        <v>33</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>92</v>
@@ -1213,10 +1241,47 @@
         <v>1</v>
       </c>
     </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E27" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" s="2">
+        <v>1</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T39">
-    <sortCondition descending="1" ref="E2:E39"/>
-    <sortCondition ref="A2:A39"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T40">
+    <sortCondition descending="1" ref="E2:E40"/>
+    <sortCondition ref="A2:A40"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="D8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -1225,15 +1290,17 @@
     <hyperlink ref="D19" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="D20" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="D21" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="D26" r:id="rId7" xr:uid="{66908C88-96C6-45C0-8372-4B5EE9147081}"/>
-    <hyperlink ref="D25" r:id="rId8" xr:uid="{104257D5-4707-4FB8-93B9-28BEF0F71FF7}"/>
+    <hyperlink ref="D27" r:id="rId7" xr:uid="{66908C88-96C6-45C0-8372-4B5EE9147081}"/>
+    <hyperlink ref="D26" r:id="rId8" xr:uid="{104257D5-4707-4FB8-93B9-28BEF0F71FF7}"/>
     <hyperlink ref="D4" r:id="rId9" xr:uid="{3DEAF3FD-C05E-4A22-99A8-24837B8931F2}"/>
     <hyperlink ref="D16" r:id="rId10" xr:uid="{530544EC-9426-44E0-BB29-E6FEEFED4C0A}"/>
-    <hyperlink ref="D24" r:id="rId11" xr:uid="{39D7A9DF-2FEF-48DC-B88C-BC52F9C79070}"/>
-    <hyperlink ref="D23" r:id="rId12" xr:uid="{F9508FD9-029B-4022-9204-E6F0CED0E479}"/>
+    <hyperlink ref="D25" r:id="rId11" xr:uid="{39D7A9DF-2FEF-48DC-B88C-BC52F9C79070}"/>
+    <hyperlink ref="D24" r:id="rId12" xr:uid="{F9508FD9-029B-4022-9204-E6F0CED0E479}"/>
     <hyperlink ref="D13" r:id="rId13" xr:uid="{37E91FF0-D1DA-4157-90CE-2B8A88B0CEDD}"/>
+    <hyperlink ref="D23" r:id="rId14" xr:uid="{840149A0-8A17-4345-9FE4-A897EF5533D8}"/>
+    <hyperlink ref="D28" r:id="rId15" xr:uid="{B145FFDB-E550-477C-85F2-4E1AEBFE976A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId14"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>